<commit_message>
Agrega validacion robusta a config_loader.py, sube capturas/ y agrega CI con GitHub Actions
</commit_message>
<xml_diff>
--- a/reports/report.xlsx
+++ b/reports/report.xlsx
@@ -475,31 +475,31 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.002862101691254651</v>
+        <v>0.794997116864921</v>
       </c>
       <c r="C2" t="n">
-        <v>0.004539473684210526</v>
+        <v>0.7794736842105262</v>
       </c>
       <c r="D2" t="n">
-        <v>0.004547276200839227</v>
+        <v>0.7812004932368943</v>
       </c>
       <c r="E2" t="n">
-        <v>0.003611111111111111</v>
+        <v>0.818912037037037</v>
       </c>
       <c r="F2" t="n">
-        <v>0.003594679752959329</v>
+        <v>0.8214135048235172</v>
       </c>
       <c r="G2" t="n">
-        <v>0.001969696969696969</v>
+        <v>0.6685037878787878</v>
       </c>
       <c r="H2" t="n">
-        <v>0.001974879518788985</v>
+        <v>0.6690024488426775</v>
       </c>
       <c r="I2" t="n">
-        <v>0.001328125</v>
+        <v>0.9130989583333334</v>
       </c>
       <c r="J2" t="n">
-        <v>0.001367042829253232</v>
+        <v>0.9181086456706462</v>
       </c>
     </row>
     <row r="3">
@@ -507,31 +507,31 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>0.002824305970893142</v>
+        <v>0.743058116804005</v>
       </c>
       <c r="C3" t="n">
-        <v>0.004495614035087719</v>
+        <v>0.7285087719298246</v>
       </c>
       <c r="D3" t="n">
-        <v>0.004461857854675625</v>
+        <v>0.7304759952099446</v>
       </c>
       <c r="E3" t="n">
-        <v>0.003541666666666667</v>
+        <v>0.7657407407407407</v>
       </c>
       <c r="F3" t="n">
-        <v>0.003563433569016916</v>
+        <v>0.768025151031335</v>
       </c>
       <c r="G3" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6247537878787879</v>
       </c>
       <c r="H3" t="n">
-        <v>0.001930235969886004</v>
+        <v>0.6254426841275572</v>
       </c>
       <c r="I3" t="n">
-        <v>0.001328125</v>
+        <v>0.8532291666666668</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0013398538334174</v>
+        <v>0.8578459571752154</v>
       </c>
     </row>
     <row r="4">
@@ -539,31 +539,31 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>0.002818823514752791</v>
+        <v>0.7178200660663654</v>
       </c>
       <c r="C4" t="n">
-        <v>0.004473684210526315</v>
+        <v>0.7039912280701754</v>
       </c>
       <c r="D4" t="n">
-        <v>0.004473062902326615</v>
+        <v>0.7051166665796061</v>
       </c>
       <c r="E4" t="n">
-        <v>0.003541666666666666</v>
+        <v>0.7394907407407408</v>
       </c>
       <c r="F4" t="n">
-        <v>0.003538596557359427</v>
+        <v>0.7416142700451775</v>
       </c>
       <c r="G4" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6035795454545455</v>
       </c>
       <c r="H4" t="n">
-        <v>0.001933043453298455</v>
+        <v>0.6039662820856428</v>
       </c>
       <c r="I4" t="n">
-        <v>0.001328125</v>
+        <v>0.82421875</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001331168786821838</v>
+        <v>0.8282256768055352</v>
       </c>
     </row>
     <row r="5">
@@ -571,31 +571,31 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>0.002830093007930179</v>
+        <v>0.7522948889941078</v>
       </c>
       <c r="C5" t="n">
-        <v>0.004495614035087719</v>
+        <v>0.7374999999999998</v>
       </c>
       <c r="D5" t="n">
-        <v>0.004514331156368383</v>
+        <v>0.7391182972835246</v>
       </c>
       <c r="E5" t="n">
-        <v>0.003564814814814815</v>
+        <v>0.7751620370370372</v>
       </c>
       <c r="F5" t="n">
-        <v>0.003555106172834477</v>
+        <v>0.7771150146059986</v>
       </c>
       <c r="G5" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6324810606060606</v>
       </c>
       <c r="H5" t="n">
-        <v>0.001948077658569888</v>
+        <v>0.6331887640452973</v>
       </c>
       <c r="I5" t="n">
-        <v>0.001328125</v>
+        <v>0.8640364583333334</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001340069636282748</v>
+        <v>0.8684163490936426</v>
       </c>
     </row>
     <row r="6">
@@ -603,31 +603,31 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>0.002818823514752791</v>
+        <v>0.7736332589879055</v>
       </c>
       <c r="C6" t="n">
-        <v>0.004473684210526315</v>
+        <v>0.7586184210526317</v>
       </c>
       <c r="D6" t="n">
-        <v>0.004498208944027497</v>
+        <v>0.7600540789229133</v>
       </c>
       <c r="E6" t="n">
-        <v>0.003541666666666666</v>
+        <v>0.7969444444444445</v>
       </c>
       <c r="F6" t="n">
-        <v>0.003544894522859754</v>
+        <v>0.7998374833180484</v>
       </c>
       <c r="G6" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6504545454545455</v>
       </c>
       <c r="H6" t="n">
-        <v>0.001927971184894132</v>
+        <v>0.6510396019466144</v>
       </c>
       <c r="I6" t="n">
-        <v>0.001328125</v>
+        <v>0.8885156250000001</v>
       </c>
       <c r="J6" t="n">
-        <v>0.001340518134537165</v>
+        <v>0.8927984319253325</v>
       </c>
     </row>
     <row r="7">
@@ -635,31 +635,31 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>0.002834827856415028</v>
+        <v>0.7427752546019406</v>
       </c>
       <c r="C7" t="n">
-        <v>0.004495614035087719</v>
+        <v>0.7283114035087719</v>
       </c>
       <c r="D7" t="n">
-        <v>0.004498299589122704</v>
+        <v>0.7301891503063107</v>
       </c>
       <c r="E7" t="n">
-        <v>0.003564814814814815</v>
+        <v>0.7652777777777778</v>
       </c>
       <c r="F7" t="n">
-        <v>0.003571146224246369</v>
+        <v>0.7674797017465962</v>
       </c>
       <c r="G7" t="n">
-        <v>0.001950757575757576</v>
+        <v>0.6244128787878788</v>
       </c>
       <c r="H7" t="n">
-        <v>0.00193920847091722</v>
+        <v>0.6252748877960754</v>
       </c>
       <c r="I7" t="n">
-        <v>0.001328125</v>
+        <v>0.8530989583333335</v>
       </c>
       <c r="J7" t="n">
-        <v>0.001335534402685642</v>
+        <v>0.8571143458241683</v>
       </c>
     </row>
     <row r="8">
@@ -667,31 +667,31 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>0.002818823514752791</v>
+        <v>0.7256316280956495</v>
       </c>
       <c r="C8" t="n">
-        <v>0.004473684210526315</v>
+        <v>0.7102850877192982</v>
       </c>
       <c r="D8" t="n">
-        <v>0.004486626975020868</v>
+        <v>0.7121292811623758</v>
       </c>
       <c r="E8" t="n">
-        <v>0.003541666666666666</v>
+        <v>0.7471064814814815</v>
       </c>
       <c r="F8" t="n">
-        <v>0.003539315173024845</v>
+        <v>0.749613389684642</v>
       </c>
       <c r="G8" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6106818181818182</v>
       </c>
       <c r="H8" t="n">
-        <v>0.001931213240125928</v>
+        <v>0.6112943632894704</v>
       </c>
       <c r="I8" t="n">
-        <v>0.001328125</v>
+        <v>0.8344531250000001</v>
       </c>
       <c r="J8" t="n">
-        <v>0.001325329212612318</v>
+        <v>0.8381464743990288</v>
       </c>
     </row>
     <row r="9">
@@ -699,31 +699,31 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0.002824305970893142</v>
+        <v>0.7227980670188729</v>
       </c>
       <c r="C9" t="n">
-        <v>0.004495614035087719</v>
+        <v>0.7086622807017544</v>
       </c>
       <c r="D9" t="n">
-        <v>0.004512725091532843</v>
+        <v>0.709996963796984</v>
       </c>
       <c r="E9" t="n">
-        <v>0.003541666666666667</v>
+        <v>0.7447222222222222</v>
       </c>
       <c r="F9" t="n">
-        <v>0.003569864322414455</v>
+        <v>0.7467105001142957</v>
       </c>
       <c r="G9" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6078598484848485</v>
       </c>
       <c r="H9" t="n">
-        <v>0.001922992791549401</v>
+        <v>0.608256420982542</v>
       </c>
       <c r="I9" t="n">
-        <v>0.001328125</v>
+        <v>0.8299479166666668</v>
       </c>
       <c r="J9" t="n">
-        <v>0.001336716146495776</v>
+        <v>0.8347797987958032</v>
       </c>
     </row>
     <row r="10">
@@ -731,31 +731,31 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>0.002824305970893142</v>
+        <v>0.6759114721779196</v>
       </c>
       <c r="C10" t="n">
-        <v>0.004495614035087719</v>
+        <v>0.6630482456140351</v>
       </c>
       <c r="D10" t="n">
-        <v>0.004502039000950194</v>
+        <v>0.6640880470974821</v>
       </c>
       <c r="E10" t="n">
-        <v>0.003541666666666667</v>
+        <v>0.6966203703703705</v>
       </c>
       <c r="F10" t="n">
-        <v>0.003542809445618163</v>
+        <v>0.6986041976505177</v>
       </c>
       <c r="G10" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.5681439393939394</v>
       </c>
       <c r="H10" t="n">
-        <v>0.00193678959691049</v>
+        <v>0.5689861885086105</v>
       </c>
       <c r="I10" t="n">
-        <v>0.001328125</v>
+        <v>0.7758333333333334</v>
       </c>
       <c r="J10" t="n">
-        <v>0.001332854252695751</v>
+        <v>0.779485327765414</v>
       </c>
     </row>
     <row r="11">
@@ -763,31 +763,31 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>0.002834827856415027</v>
+        <v>0.6912420220571948</v>
       </c>
       <c r="C11" t="n">
-        <v>0.004495614035087719</v>
+        <v>0.6781359649122807</v>
       </c>
       <c r="D11" t="n">
-        <v>0.004546775676008904</v>
+        <v>0.6798931430879769</v>
       </c>
       <c r="E11" t="n">
-        <v>0.003564814814814815</v>
+        <v>0.7119907407407409</v>
       </c>
       <c r="F11" t="n">
-        <v>0.003563829644736449</v>
+        <v>0.7144851688858076</v>
       </c>
       <c r="G11" t="n">
-        <v>0.001950757575757576</v>
+        <v>0.5811174242424241</v>
       </c>
       <c r="H11" t="n">
-        <v>0.001955311976620059</v>
+        <v>0.5815307015682706</v>
       </c>
       <c r="I11" t="n">
-        <v>0.001328125</v>
+        <v>0.7937239583333334</v>
       </c>
       <c r="J11" t="n">
-        <v>0.001324808317032929</v>
+        <v>0.7974083023557503</v>
       </c>
     </row>
     <row r="12">
@@ -795,31 +795,31 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>0.002829788427033493</v>
+        <v>0.7326668480307461</v>
       </c>
       <c r="C12" t="n">
-        <v>0.004517543859649122</v>
+        <v>0.7182236842105263</v>
       </c>
       <c r="D12" t="n">
-        <v>0.004550578895201074</v>
+        <v>0.719349642065733</v>
       </c>
       <c r="E12" t="n">
-        <v>0.003541666666666666</v>
+        <v>0.7547685185185186</v>
       </c>
       <c r="F12" t="n">
-        <v>0.003595601007044028</v>
+        <v>0.7568776884963787</v>
       </c>
       <c r="G12" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.616060606060606</v>
       </c>
       <c r="H12" t="n">
-        <v>0.001935170229115032</v>
+        <v>0.6165798160509265</v>
       </c>
       <c r="I12" t="n">
-        <v>0.001328125</v>
+        <v>0.8416145833333333</v>
       </c>
       <c r="J12" t="n">
-        <v>0.001313314427766617</v>
+        <v>0.8455687525171458</v>
       </c>
     </row>
     <row r="13">
@@ -827,31 +827,31 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>0.002818823514752791</v>
+        <v>0.6655867750974659</v>
       </c>
       <c r="C13" t="n">
-        <v>0.004473684210526315</v>
+        <v>0.6529605263157895</v>
       </c>
       <c r="D13" t="n">
-        <v>0.004466786446201828</v>
+        <v>0.6545388971288967</v>
       </c>
       <c r="E13" t="n">
-        <v>0.003541666666666666</v>
+        <v>0.6857407407407408</v>
       </c>
       <c r="F13" t="n">
-        <v>0.003530166682055324</v>
+        <v>0.6881167064905861</v>
       </c>
       <c r="G13" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.559375</v>
       </c>
       <c r="H13" t="n">
-        <v>0.001927700336119242</v>
+        <v>0.5601349759402698</v>
       </c>
       <c r="I13" t="n">
-        <v>0.001328125</v>
+        <v>0.7642708333333335</v>
       </c>
       <c r="J13" t="n">
-        <v>0.001341770741413906</v>
+        <v>0.7681315277906795</v>
       </c>
     </row>
     <row r="14">
@@ -859,31 +859,31 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>0.002818823514752791</v>
+        <v>0.6753350286029152</v>
       </c>
       <c r="C14" t="n">
-        <v>0.004473684210526316</v>
+        <v>0.6622368421052631</v>
       </c>
       <c r="D14" t="n">
-        <v>0.004543293127548864</v>
+        <v>0.6632329981685018</v>
       </c>
       <c r="E14" t="n">
-        <v>0.003541666666666666</v>
+        <v>0.6960185185185185</v>
       </c>
       <c r="F14" t="n">
-        <v>0.003531396334506742</v>
+        <v>0.6976512830955027</v>
       </c>
       <c r="G14" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.5679545454545455</v>
       </c>
       <c r="H14" t="n">
-        <v>0.001932552758716407</v>
+        <v>0.5685761237913486</v>
       </c>
       <c r="I14" t="n">
-        <v>0.001328125</v>
+        <v>0.7751302083333336</v>
       </c>
       <c r="J14" t="n">
-        <v>0.00134535187200658</v>
+        <v>0.7793843347013784</v>
       </c>
     </row>
     <row r="15">
@@ -891,31 +891,31 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>0.002824305970893142</v>
+        <v>0.7781673782783982</v>
       </c>
       <c r="C15" t="n">
-        <v>0.004495614035087719</v>
+        <v>0.7627631578947369</v>
       </c>
       <c r="D15" t="n">
-        <v>0.004534080343438251</v>
+        <v>0.7644485332855699</v>
       </c>
       <c r="E15" t="n">
-        <v>0.003541666666666667</v>
+        <v>0.8016203703703705</v>
       </c>
       <c r="F15" t="n">
-        <v>0.003561299668201468</v>
+        <v>0.8036778177822469</v>
       </c>
       <c r="G15" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6542234848484848</v>
       </c>
       <c r="H15" t="n">
-        <v>0.001931128610981311</v>
+        <v>0.6549279639104861</v>
       </c>
       <c r="I15" t="n">
-        <v>0.001328125</v>
+        <v>0.8940625000000002</v>
       </c>
       <c r="J15" t="n">
-        <v>0.001336838013247147</v>
+        <v>0.8980035425675161</v>
       </c>
     </row>
     <row r="16">
@@ -923,31 +923,31 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>0.00283557546407053</v>
+        <v>0.7221626420454546</v>
       </c>
       <c r="C16" t="n">
-        <v>0.004517543859649122</v>
+        <v>0.7079166666666666</v>
       </c>
       <c r="D16" t="n">
-        <v>0.004524658051337882</v>
+        <v>0.7095502974641238</v>
       </c>
       <c r="E16" t="n">
-        <v>0.003564814814814815</v>
+        <v>0.7441666666666668</v>
       </c>
       <c r="F16" t="n">
-        <v>0.003578659593988857</v>
+        <v>0.7460262441655076</v>
       </c>
       <c r="G16" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6073484848484848</v>
       </c>
       <c r="H16" t="n">
-        <v>0.00194885736437244</v>
+        <v>0.6078208805534886</v>
       </c>
       <c r="I16" t="n">
-        <v>0.001328125</v>
+        <v>0.8292187500000001</v>
       </c>
       <c r="J16" t="n">
-        <v>0.001322516092427913</v>
+        <v>0.8337320800002442</v>
       </c>
     </row>
     <row r="17">
@@ -955,31 +955,31 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>0.002818823514752791</v>
+        <v>0.698399081273259</v>
       </c>
       <c r="C17" t="n">
-        <v>0.004473684210526315</v>
+        <v>0.6848684210526317</v>
       </c>
       <c r="D17" t="n">
-        <v>0.004470337681003252</v>
+        <v>0.6864326685133464</v>
       </c>
       <c r="E17" t="n">
-        <v>0.003541666666666666</v>
+        <v>0.7197222222222223</v>
       </c>
       <c r="F17" t="n">
-        <v>0.003544570907326376</v>
+        <v>0.722012873328813</v>
       </c>
       <c r="G17" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.5872348484848485</v>
       </c>
       <c r="H17" t="n">
-        <v>0.001941175205342693</v>
+        <v>0.5879946106422034</v>
       </c>
       <c r="I17" t="n">
-        <v>0.001328125</v>
+        <v>0.8017708333333332</v>
       </c>
       <c r="J17" t="n">
-        <v>0.001327257397721067</v>
+        <v>0.8058148281269341</v>
       </c>
     </row>
     <row r="18">
@@ -987,31 +987,31 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>0.002818823514752791</v>
+        <v>0.8165639329146731</v>
       </c>
       <c r="C18" t="n">
-        <v>0.004473684210526315</v>
+        <v>0.8007017543859649</v>
       </c>
       <c r="D18" t="n">
-        <v>0.004463352343812943</v>
+        <v>0.8024409339107582</v>
       </c>
       <c r="E18" t="n">
-        <v>0.003541666666666666</v>
+        <v>0.8410416666666668</v>
       </c>
       <c r="F18" t="n">
-        <v>0.003535984756019972</v>
+        <v>0.8438326220003554</v>
       </c>
       <c r="G18" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6864393939393938</v>
       </c>
       <c r="H18" t="n">
-        <v>0.001933439906995467</v>
+        <v>0.6871717708413293</v>
       </c>
       <c r="I18" t="n">
-        <v>0.001328125</v>
+        <v>0.9380729166666667</v>
       </c>
       <c r="J18" t="n">
-        <v>0.001341031679793551</v>
+        <v>0.942633409011317</v>
       </c>
     </row>
     <row r="19">
@@ -1019,31 +1019,31 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>0.002834827856415028</v>
+        <v>0.7957655675449673</v>
       </c>
       <c r="C19" t="n">
-        <v>0.004495614035087719</v>
+        <v>0.7799122807017544</v>
       </c>
       <c r="D19" t="n">
-        <v>0.004516316047999788</v>
+        <v>0.7817653902974183</v>
       </c>
       <c r="E19" t="n">
-        <v>0.003564814814814815</v>
+        <v>0.8200462962962964</v>
       </c>
       <c r="F19" t="n">
-        <v>0.003559049361763219</v>
+        <v>0.8221499368804818</v>
       </c>
       <c r="G19" t="n">
-        <v>0.001950757575757576</v>
+        <v>0.6692234848484848</v>
       </c>
       <c r="H19" t="n">
-        <v>0.001946650161773281</v>
+        <v>0.6700784962282591</v>
       </c>
       <c r="I19" t="n">
-        <v>0.001328125</v>
+        <v>0.9138802083333335</v>
       </c>
       <c r="J19" t="n">
-        <v>0.001359310029473641</v>
+        <v>0.9191883505349165</v>
       </c>
     </row>
     <row r="20">
@@ -1051,31 +1051,31 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>0.002818823514752791</v>
+        <v>0.7372588688419281</v>
       </c>
       <c r="C20" t="n">
-        <v>0.004473684210526315</v>
+        <v>0.7224561403508771</v>
       </c>
       <c r="D20" t="n">
-        <v>0.004489124421495887</v>
+        <v>0.7239907699474518</v>
       </c>
       <c r="E20" t="n">
-        <v>0.003541666666666666</v>
+        <v>0.7594675925925928</v>
       </c>
       <c r="F20" t="n">
-        <v>0.003537277815853038</v>
+        <v>0.7612716573449031</v>
       </c>
       <c r="G20" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6199242424242425</v>
       </c>
       <c r="H20" t="n">
-        <v>0.001929628529324619</v>
+        <v>0.6203457518008015</v>
       </c>
       <c r="I20" t="n">
-        <v>0.001328125</v>
+        <v>0.8471874999999999</v>
       </c>
       <c r="J20" t="n">
-        <v>0.00130563088638905</v>
+        <v>0.850876464053026</v>
       </c>
     </row>
     <row r="21">
@@ -1083,31 +1083,31 @@
         <v>20</v>
       </c>
       <c r="B21" t="n">
-        <v>0.002840310312555378</v>
+        <v>0.726734778569688</v>
       </c>
       <c r="C21" t="n">
-        <v>0.004517543859649122</v>
+        <v>0.710877192982456</v>
       </c>
       <c r="D21" t="n">
-        <v>0.004573083499145003</v>
+        <v>0.712626925678527</v>
       </c>
       <c r="E21" t="n">
-        <v>0.003564814814814815</v>
+        <v>0.7481712962962963</v>
       </c>
       <c r="F21" t="n">
-        <v>0.003592147186137895</v>
+        <v>0.7502605163375154</v>
       </c>
       <c r="G21" t="n">
-        <v>0.001950757575757576</v>
+        <v>0.6114583333333333</v>
       </c>
       <c r="H21" t="n">
-        <v>0.001949432579093258</v>
+        <v>0.6120567520055986</v>
       </c>
       <c r="I21" t="n">
-        <v>0.001328125</v>
+        <v>0.8364322916666667</v>
       </c>
       <c r="J21" t="n">
-        <v>0.001380142917024929</v>
+        <v>0.8403099968905795</v>
       </c>
     </row>
     <row r="22">
@@ -1115,31 +1115,31 @@
         <v>21</v>
       </c>
       <c r="B22" t="n">
-        <v>0.002846540376351232</v>
+        <v>0.7594282082059631</v>
       </c>
       <c r="C22" t="n">
-        <v>0.004561403508771929</v>
+        <v>0.7450657894736842</v>
       </c>
       <c r="D22" t="n">
-        <v>0.004622459046522609</v>
+        <v>0.7464280394882944</v>
       </c>
       <c r="E22" t="n">
-        <v>0.003564814814814815</v>
+        <v>0.7823842592592593</v>
       </c>
       <c r="F22" t="n">
-        <v>0.003628771729444106</v>
+        <v>0.7850235289118851</v>
       </c>
       <c r="G22" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6384659090909091</v>
       </c>
       <c r="H22" t="n">
-        <v>0.001958470738043501</v>
+        <v>0.6392278398828721</v>
       </c>
       <c r="I22" t="n">
-        <v>0.001328125</v>
+        <v>0.871796875</v>
       </c>
       <c r="J22" t="n">
-        <v>0.001334146328078652</v>
+        <v>0.8762173039374114</v>
       </c>
     </row>
     <row r="23">
@@ -1147,31 +1147,31 @@
         <v>22</v>
       </c>
       <c r="B23" t="n">
-        <v>0.002818823514752791</v>
+        <v>0.5241686602870814</v>
       </c>
       <c r="C23" t="n">
-        <v>0.004473684210526315</v>
+        <v>0.5143640350877193</v>
       </c>
       <c r="D23" t="n">
-        <v>0.004469822433497361</v>
+        <v>0.5157062852069344</v>
       </c>
       <c r="E23" t="n">
-        <v>0.003541666666666666</v>
+        <v>0.5402083333333334</v>
       </c>
       <c r="F23" t="n">
-        <v>0.003541396215189097</v>
+        <v>0.5418523110491404</v>
       </c>
       <c r="G23" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.4406439393939394</v>
       </c>
       <c r="H23" t="n">
-        <v>0.001930429165784039</v>
+        <v>0.4410105065711279</v>
       </c>
       <c r="I23" t="n">
-        <v>0.001328125</v>
+        <v>0.6014583333333334</v>
       </c>
       <c r="J23" t="n">
-        <v>0.001355682724019972</v>
+        <v>0.6044184290835805</v>
       </c>
     </row>
     <row r="24">
@@ -1179,31 +1179,31 @@
         <v>23</v>
       </c>
       <c r="B24" t="n">
-        <v>0.002824305970893142</v>
+        <v>0.7569425165858142</v>
       </c>
       <c r="C24" t="n">
-        <v>0.004495614035087719</v>
+        <v>0.7418859649122808</v>
       </c>
       <c r="D24" t="n">
-        <v>0.004475804052565957</v>
+        <v>0.7435934488368107</v>
       </c>
       <c r="E24" t="n">
-        <v>0.003541666666666667</v>
+        <v>0.7797453703703704</v>
       </c>
       <c r="F24" t="n">
-        <v>0.003577706681019858</v>
+        <v>0.7819160696601186</v>
       </c>
       <c r="G24" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6364772727272727</v>
       </c>
       <c r="H24" t="n">
-        <v>0.001926360204594787</v>
+        <v>0.6370741864659217</v>
       </c>
       <c r="I24" t="n">
-        <v>0.001328125</v>
+        <v>0.8696614583333334</v>
       </c>
       <c r="J24" t="n">
-        <v>0.001327571734300648</v>
+        <v>0.8734727851007797</v>
       </c>
     </row>
     <row r="25">
@@ -1211,31 +1211,31 @@
         <v>24</v>
       </c>
       <c r="B25" t="n">
-        <v>0.002818823514752791</v>
+        <v>0.7610123265273349</v>
       </c>
       <c r="C25" t="n">
-        <v>0.004473684210526315</v>
+        <v>0.7459429824561404</v>
       </c>
       <c r="D25" t="n">
-        <v>0.00445780853381604</v>
+        <v>0.7477331076216825</v>
       </c>
       <c r="E25" t="n">
-        <v>0.003541666666666666</v>
+        <v>0.7840509259259261</v>
       </c>
       <c r="F25" t="n">
-        <v>0.003534388526529534</v>
+        <v>0.7860959007473209</v>
       </c>
       <c r="G25" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6400189393939395</v>
       </c>
       <c r="H25" t="n">
-        <v>0.001938775023124865</v>
+        <v>0.6405307801233372</v>
       </c>
       <c r="I25" t="n">
-        <v>0.001328125</v>
+        <v>0.8740364583333334</v>
       </c>
       <c r="J25" t="n">
-        <v>0.001329556883361442</v>
+        <v>0.8789990772774673</v>
       </c>
     </row>
     <row r="26">
@@ -1243,31 +1243,31 @@
         <v>25</v>
       </c>
       <c r="B26" t="n">
-        <v>0.002824305970893142</v>
+        <v>0.8031338743797625</v>
       </c>
       <c r="C26" t="n">
-        <v>0.004495614035087719</v>
+        <v>0.7872587719298244</v>
       </c>
       <c r="D26" t="n">
-        <v>0.004528629473577868</v>
+        <v>0.7887512614943663</v>
       </c>
       <c r="E26" t="n">
-        <v>0.003541666666666667</v>
+        <v>0.8274074074074074</v>
       </c>
       <c r="F26" t="n">
-        <v>0.003565753663521343</v>
+        <v>0.8294609184714243</v>
       </c>
       <c r="G26" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6754734848484848</v>
       </c>
       <c r="H26" t="n">
-        <v>0.001931655637779632</v>
+        <v>0.6760008833730503</v>
       </c>
       <c r="I26" t="n">
-        <v>0.001328125</v>
+        <v>0.9223958333333335</v>
       </c>
       <c r="J26" t="n">
-        <v>0.001315746041186124</v>
+        <v>0.9272276350042975</v>
       </c>
     </row>
     <row r="27">
@@ -1275,31 +1275,31 @@
         <v>26</v>
       </c>
       <c r="B27" t="n">
-        <v>0.002818823514752791</v>
+        <v>0.7450115221568758</v>
       </c>
       <c r="C27" t="n">
-        <v>0.004473684210526315</v>
+        <v>0.7305482456140352</v>
       </c>
       <c r="D27" t="n">
-        <v>0.004469644980519109</v>
+        <v>0.7319322830397029</v>
       </c>
       <c r="E27" t="n">
-        <v>0.003541666666666666</v>
+        <v>0.7671990740740741</v>
       </c>
       <c r="F27" t="n">
-        <v>0.003531578592421947</v>
+        <v>0.769740004431177</v>
       </c>
       <c r="G27" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6262310606060606</v>
       </c>
       <c r="H27" t="n">
-        <v>0.00193055496823998</v>
+        <v>0.6267271095728436</v>
       </c>
       <c r="I27" t="n">
-        <v>0.001328125</v>
+        <v>0.8560677083333335</v>
       </c>
       <c r="J27" t="n">
-        <v>0.001353874737744783</v>
+        <v>0.8592809386762347</v>
       </c>
     </row>
     <row r="28">
@@ -1307,31 +1307,31 @@
         <v>27</v>
       </c>
       <c r="B28" t="n">
-        <v>0.00283557546407053</v>
+        <v>0.7535389669723551</v>
       </c>
       <c r="C28" t="n">
-        <v>0.004517543859649122</v>
+        <v>0.7385087719298244</v>
       </c>
       <c r="D28" t="n">
-        <v>0.004516038827569376</v>
+        <v>0.740226284214217</v>
       </c>
       <c r="E28" t="n">
-        <v>0.003564814814814815</v>
+        <v>0.7763194444444446</v>
       </c>
       <c r="F28" t="n">
-        <v>0.00360455538419493</v>
+        <v>0.7781556426461904</v>
       </c>
       <c r="G28" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6335984848484848</v>
       </c>
       <c r="H28" t="n">
-        <v>0.001950387347443083</v>
+        <v>0.6341725889932467</v>
       </c>
       <c r="I28" t="n">
-        <v>0.001328125</v>
+        <v>0.8657291666666668</v>
       </c>
       <c r="J28" t="n">
-        <v>0.00132891129504907</v>
+        <v>0.8698639295604677</v>
       </c>
     </row>
     <row r="29">
@@ -1339,31 +1339,31 @@
         <v>28</v>
       </c>
       <c r="B29" t="n">
-        <v>0.002840310312555378</v>
+        <v>0.7337284993576112</v>
       </c>
       <c r="C29" t="n">
-        <v>0.004517543859649122</v>
+        <v>0.7194078947368421</v>
       </c>
       <c r="D29" t="n">
-        <v>0.004510954844815732</v>
+        <v>0.7208508054371449</v>
       </c>
       <c r="E29" t="n">
-        <v>0.003564814814814815</v>
+        <v>0.7558564814814815</v>
       </c>
       <c r="F29" t="n">
-        <v>0.003601245318371612</v>
+        <v>0.7585343308265318</v>
       </c>
       <c r="G29" t="n">
-        <v>0.001950757575757576</v>
+        <v>0.6168371212121211</v>
       </c>
       <c r="H29" t="n">
-        <v>0.001957903845432647</v>
+        <v>0.6174549330250652</v>
       </c>
       <c r="I29" t="n">
-        <v>0.001328125</v>
+        <v>0.8428125000000002</v>
       </c>
       <c r="J29" t="n">
-        <v>0.001372584023602097</v>
+        <v>0.8469196686743889</v>
       </c>
     </row>
     <row r="30">
@@ -1371,31 +1371,31 @@
         <v>29</v>
       </c>
       <c r="B30" t="n">
-        <v>0.002824305970893142</v>
+        <v>0.7954631014088251</v>
       </c>
       <c r="C30" t="n">
-        <v>0.004495614035087719</v>
+        <v>0.7800657894736842</v>
       </c>
       <c r="D30" t="n">
-        <v>0.004502527568590701</v>
+        <v>0.7816053861970222</v>
       </c>
       <c r="E30" t="n">
-        <v>0.003541666666666667</v>
+        <v>0.8193055555555555</v>
       </c>
       <c r="F30" t="n">
-        <v>0.003570345241719626</v>
+        <v>0.8223648862572815</v>
       </c>
       <c r="G30" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6687310606060606</v>
       </c>
       <c r="H30" t="n">
-        <v>0.00193213122096411</v>
+        <v>0.6691354579980371</v>
       </c>
       <c r="I30" t="n">
-        <v>0.001328125</v>
+        <v>0.9137500000000002</v>
       </c>
       <c r="J30" t="n">
-        <v>0.001320087687864165</v>
+        <v>0.9185327622419547</v>
       </c>
     </row>
     <row r="31">
@@ -1403,31 +1403,31 @@
         <v>30</v>
       </c>
       <c r="B31" t="n">
-        <v>0.002829788427033493</v>
+        <v>0.7405616783238083</v>
       </c>
       <c r="C31" t="n">
-        <v>0.004517543859649122</v>
+        <v>0.7263157894736841</v>
       </c>
       <c r="D31" t="n">
-        <v>0.004511055508015923</v>
+        <v>0.7278335294039695</v>
       </c>
       <c r="E31" t="n">
-        <v>0.003541666666666666</v>
+        <v>0.7628935185185186</v>
       </c>
       <c r="F31" t="n">
-        <v>0.003569662417417489</v>
+        <v>0.7655117755422621</v>
       </c>
       <c r="G31" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6225946969696969</v>
       </c>
       <c r="H31" t="n">
-        <v>0.001920917113852812</v>
+        <v>0.6233312083467225</v>
       </c>
       <c r="I31" t="n">
-        <v>0.001328125</v>
+        <v>0.8504427083333334</v>
       </c>
       <c r="J31" t="n">
-        <v>0.001324243561507532</v>
+        <v>0.8542282580562782</v>
       </c>
     </row>
   </sheetData>
@@ -1503,31 +1503,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.165306643847643</v>
+        <v>349.3600941139053</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>16.58775616802892</v>
       </c>
       <c r="D2" t="n">
-        <v>477.8346933561523</v>
+        <v>114.0521497180657</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>206</v>
+        <v>33120</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>0.9654421746499398</v>
       </c>
       <c r="H2" t="n">
-        <v>0.004517543859649122</v>
+        <v>0.7536543028966302</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>0.9982217667801923</v>
       </c>
       <c r="J2" t="n">
-        <v>0.004517543859649122</v>
+        <v>0.7263157894736841</v>
       </c>
     </row>
     <row r="3">
@@ -1537,31 +1537,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.713437960360395</v>
+        <v>367.4456522602858</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>27.83088426286508</v>
       </c>
       <c r="D3" t="n">
-        <v>478.2760651404432</v>
+        <v>69.98860406232359</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01049689919636521</v>
+        <v>14.73485941452553</v>
       </c>
       <c r="F3" t="n">
-        <v>153</v>
+        <v>32957</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>0.9420189911190311</v>
       </c>
       <c r="H3" t="n">
-        <v>0.003587962962962963</v>
+        <v>0.8126015699553836</v>
       </c>
       <c r="I3" t="n">
-        <v>0.9870967741935484</v>
+        <v>0.9966131422177871</v>
       </c>
       <c r="J3" t="n">
-        <v>0.003541666666666666</v>
+        <v>0.7628935185185186</v>
       </c>
     </row>
     <row r="4">
@@ -1571,31 +1571,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9220402146493498</v>
+        <v>299.1989800064268</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>478.8441749756712</v>
+        <v>134.9965881040019</v>
       </c>
       <c r="E4" t="n">
-        <v>0.233784809679463</v>
+        <v>45.80443188957135</v>
       </c>
       <c r="F4" t="n">
-        <v>102</v>
+        <v>32873</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6232196969696969</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0.9989971433781073</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001931818181818182</v>
+        <v>0.6225946969696969</v>
       </c>
     </row>
     <row r="5">
@@ -1605,31 +1605,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6356369095236154</v>
+        <v>410.0295638670136</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>36.47187395509383</v>
       </c>
       <c r="D5" t="n">
-        <v>479.3331840676005</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0.03117902287581487</v>
+        <v>33.49856217789259</v>
       </c>
       <c r="F5" t="n">
-        <v>51</v>
+        <v>32657</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>0.9240169292602212</v>
       </c>
       <c r="H5" t="n">
-        <v>0.001328125</v>
+        <v>0.9250258910490394</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0.9949728840411919</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001328125</v>
+        <v>0.8504427083333334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>